<commit_message>
scg case study: ingest 8 Mondays of Brink hourly reports + rebuild Excel
Bobby manually downloaded Mondays Mar 16 → Apr 27 from Brink admin5.parpos.com.
ingest_brink_downloads.py detects M/D/YYYY date headers and files each PDF to
data/raw/parbrink/2065/{date}/. Analyzer ran with 5-Monday overlap vs Teamworx
forecast captures. Excel: 5 day-detail tabs + Summary.
</commit_message>
<xml_diff>
--- a/data/case-studies/teamworx-forecast-accuracy/Teamworx_Forecast_vs_Brink_Actual_2065.xlsx
+++ b/data/case-studies/teamworx-forecast-accuracy/Teamworx_Forecast_vs_Brink_Actual_2065.xlsx
@@ -1,14 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2026-04-27" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-03-30" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-04-06" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-04-13" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-04-20" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-04-27" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:U8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -550,37 +554,193 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>3983</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>3909.06</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>-73.94000000000005</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>-0.01856389656038164</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>7PM</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>12PM</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>12PM (+61%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>4407</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>3801.8</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>-605.2000000000003</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>-0.137326979804856</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>6PM</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>7PM</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>2PM (-49%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>4326</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>3535.6</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>-790.4000000000001</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>-0.1827092001849284</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>7PM</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>7PM</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>4PM (-47%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>3754</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>3436.36</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>-317.6399999999999</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>-0.08461374533830578</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>6PM</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>6PM</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>9PM (-71%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>2026-04-27</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C8" s="3" t="n">
         <v>3964</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D8" s="3" t="n">
         <v>3805.65</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>-158.3500000000004</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>-0.03994702320888001</v>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="E8" s="4" t="n">
+        <v>-158.3499999999999</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>-0.0399470232088799</v>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>6PM</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>5PM</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>2PM (-59%)</t>
         </is>
@@ -627,6 +787,2198 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>KY-2065 — 2026-03-30 — Teamworx Forecast vs Brink Actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>6AM</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>7AM</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>8AM</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>9AM</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>10AM</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>11AM</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>12PM</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>1PM</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>2PM</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>3PM</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>4PM</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>5PM</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>6PM</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>7PM</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>8PM</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>9PM</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>10PM</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>11PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>TWX FORECAST $</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>249</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>390</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>295</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>303</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>262</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>473</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>472</v>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>468</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>535</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>345</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>191</v>
+      </c>
+      <c r="R4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>BRINK ACTUAL $</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>343.82</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>627.08</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>395.07</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>162.62</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>188.12</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>372.86</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>424.39</v>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>467.12</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>407.1</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>419.85</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>101.03</v>
+      </c>
+      <c r="R5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>VARIANCE $ (Actual−Forecast)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>94.81999999999999</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>237.08</v>
+      </c>
+      <c r="I6" s="10" t="n">
+        <v>100.07</v>
+      </c>
+      <c r="J6" s="11" t="n">
+        <v>-140.38</v>
+      </c>
+      <c r="K6" s="11" t="n">
+        <v>-73.88</v>
+      </c>
+      <c r="L6" s="11" t="n">
+        <v>-100.14</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>-47.61</v>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>-0.88</v>
+      </c>
+      <c r="O6" s="11" t="n">
+        <v>-127.9</v>
+      </c>
+      <c r="P6" s="10" t="n">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="Q6" s="11" t="n">
+        <v>-89.97</v>
+      </c>
+      <c r="R6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>VARIANCE % (Δ/Forecast)</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="n">
+        <v>0.3808032128514056</v>
+      </c>
+      <c r="H7" s="12" t="n">
+        <v>0.6078974358974361</v>
+      </c>
+      <c r="I7" s="12" t="n">
+        <v>0.3392203389830508</v>
+      </c>
+      <c r="J7" s="12" t="n">
+        <v>-0.4633003300330033</v>
+      </c>
+      <c r="K7" s="12" t="n">
+        <v>-0.2819847328244275</v>
+      </c>
+      <c r="L7" s="12" t="n">
+        <v>-0.2117124735729387</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>-0.1008686440677967</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>-0.001880341880341871</v>
+      </c>
+      <c r="O7" s="12" t="n">
+        <v>-0.2390654205607476</v>
+      </c>
+      <c r="P7" s="12" t="n">
+        <v>0.2169565217391305</v>
+      </c>
+      <c r="Q7" s="12" t="n">
+        <v>-0.4710471204188482</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>BRINK Labor Hrs</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="G9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="K9" t="n">
+        <v>7.78</v>
+      </c>
+      <c r="L9" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="M9" t="n">
+        <v>7.82</v>
+      </c>
+      <c r="N9" t="n">
+        <v>8</v>
+      </c>
+      <c r="O9" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="P9" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R9" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="S9" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>BRINK Labor $</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>13.27</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>48.37</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>65.15000000000001</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>43.54</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>66.75</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>66.75</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>66.75</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>52.28</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>90.5</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>50.7</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>90.47</v>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>92.5</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>79.67</v>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>78.5</v>
+      </c>
+      <c r="Q10" s="3" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="R10" s="3" t="n">
+        <v>57.98</v>
+      </c>
+      <c r="S10" s="3" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>BRINK Labor %</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>100</v>
+      </c>
+      <c r="D11" t="n">
+        <v>100</v>
+      </c>
+      <c r="E11" t="n">
+        <v>100</v>
+      </c>
+      <c r="F11" t="n">
+        <v>100</v>
+      </c>
+      <c r="G11" t="n">
+        <v>19.41</v>
+      </c>
+      <c r="H11" t="n">
+        <v>10.64</v>
+      </c>
+      <c r="I11" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="J11" t="n">
+        <v>32.15</v>
+      </c>
+      <c r="K11" t="n">
+        <v>48.11</v>
+      </c>
+      <c r="L11" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="M11" t="n">
+        <v>21.32</v>
+      </c>
+      <c r="N11" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="O11" t="n">
+        <v>19.57</v>
+      </c>
+      <c r="P11" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>67.01000000000001</v>
+      </c>
+      <c r="R11" t="n">
+        <v>100</v>
+      </c>
+      <c r="S11" t="n">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:S1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KY-2065 — 2026-04-06 — Teamworx Forecast vs Brink Actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>6AM</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>7AM</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>8AM</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>9AM</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>10AM</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>11AM</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>12PM</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>1PM</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>2PM</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>3PM</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>4PM</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>5PM</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>6PM</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>7PM</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>8PM</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>9PM</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>10PM</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>11PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>TWX FORECAST $</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>356</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>467</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>311</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>271</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>435</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>530</v>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>557</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>557</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>352</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>271</v>
+      </c>
+      <c r="R4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>BRINK ACTUAL $</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>378.08</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>426.07</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>270.34</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>159.24</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>296.99</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>242.98</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>316.4</v>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>472.74</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>534.53</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>306.62</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>397.81</v>
+      </c>
+      <c r="R5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>VARIANCE $ (Actual−Forecast)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>22.08</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>-40.93</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>-29.66</v>
+      </c>
+      <c r="J6" s="11" t="n">
+        <v>-151.76</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>25.99</v>
+      </c>
+      <c r="L6" s="11" t="n">
+        <v>-192.02</v>
+      </c>
+      <c r="M6" s="11" t="n">
+        <v>-213.6</v>
+      </c>
+      <c r="N6" s="11" t="n">
+        <v>-84.26000000000001</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>-22.47</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>-45.38</v>
+      </c>
+      <c r="Q6" s="10" t="n">
+        <v>126.81</v>
+      </c>
+      <c r="R6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>VARIANCE % (Δ/Forecast)</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0.06202247191011231</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>-0.08764453961456105</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>-0.09886666666666676</v>
+      </c>
+      <c r="J7" s="12" t="n">
+        <v>-0.4879742765273312</v>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>0.09590405904059043</v>
+      </c>
+      <c r="L7" s="12" t="n">
+        <v>-0.4414252873563218</v>
+      </c>
+      <c r="M7" s="12" t="n">
+        <v>-0.4030188679245283</v>
+      </c>
+      <c r="N7" s="12" t="n">
+        <v>-0.1512746858168761</v>
+      </c>
+      <c r="O7" s="5" t="n">
+        <v>-0.04034111310592464</v>
+      </c>
+      <c r="P7" s="5" t="n">
+        <v>-0.1289204545454545</v>
+      </c>
+      <c r="Q7" s="12" t="n">
+        <v>0.4679335793357934</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>BRINK Labor Hrs</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="D9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="G9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="K9" t="n">
+        <v>5.98</v>
+      </c>
+      <c r="L9" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="M9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N9" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O9" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="P9" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>7</v>
+      </c>
+      <c r="R9" t="n">
+        <v>6.95</v>
+      </c>
+      <c r="S9" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>BRINK Labor $</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>5.39</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>51.25</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>51.25</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>28.69</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>51.25</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>51.25</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>51.25</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>36.82</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>64.98</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>53.43</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>73.25</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>74.47</v>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>79.25</v>
+      </c>
+      <c r="Q10" s="3" t="n">
+        <v>79.25</v>
+      </c>
+      <c r="R10" s="3" t="n">
+        <v>78.7</v>
+      </c>
+      <c r="S10" s="3" t="n">
+        <v>8.24</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>BRINK Labor %</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>100</v>
+      </c>
+      <c r="D11" t="n">
+        <v>100</v>
+      </c>
+      <c r="E11" t="n">
+        <v>100</v>
+      </c>
+      <c r="F11" t="n">
+        <v>100</v>
+      </c>
+      <c r="G11" t="n">
+        <v>13.56</v>
+      </c>
+      <c r="H11" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="I11" t="n">
+        <v>18.96</v>
+      </c>
+      <c r="J11" t="n">
+        <v>23.12</v>
+      </c>
+      <c r="K11" t="n">
+        <v>21.88</v>
+      </c>
+      <c r="L11" t="n">
+        <v>21.99</v>
+      </c>
+      <c r="M11" t="n">
+        <v>21.33</v>
+      </c>
+      <c r="N11" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="O11" t="n">
+        <v>13.93</v>
+      </c>
+      <c r="P11" t="n">
+        <v>25.85</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>19.92</v>
+      </c>
+      <c r="R11" t="n">
+        <v>100</v>
+      </c>
+      <c r="S11" t="n">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:S1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KY-2065 — 2026-04-13 — Teamworx Forecast vs Brink Actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>6AM</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>7AM</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>8AM</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>9AM</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>10AM</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>11AM</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>12PM</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>1PM</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>2PM</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>3PM</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>4PM</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>5PM</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>6PM</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>7PM</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>8PM</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>9PM</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>10PM</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>11PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>TWX FORECAST $</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>286</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>448</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>340</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>348</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>301</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>496</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>495</v>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>490</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>561</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>361</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="R4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>BRINK ACTUAL $</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>212.36</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>279.25</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>237.64</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>266.23</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>228.47</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>262.11</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>456.53</v>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>392.45</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>569.25</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>402.72</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>228.59</v>
+      </c>
+      <c r="R5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>VARIANCE $ (Actual−Forecast)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>-73.64</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>-168.75</v>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>-102.36</v>
+      </c>
+      <c r="J6" s="11" t="n">
+        <v>-81.77</v>
+      </c>
+      <c r="K6" s="11" t="n">
+        <v>-72.53</v>
+      </c>
+      <c r="L6" s="11" t="n">
+        <v>-233.89</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>-38.47</v>
+      </c>
+      <c r="N6" s="11" t="n">
+        <v>-97.55</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>41.72</v>
+      </c>
+      <c r="Q6" s="3" t="n">
+        <v>28.59</v>
+      </c>
+      <c r="R6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>VARIANCE % (Δ/Forecast)</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="n">
+        <v>-0.2574825174825174</v>
+      </c>
+      <c r="H7" s="12" t="n">
+        <v>-0.3766741071428572</v>
+      </c>
+      <c r="I7" s="12" t="n">
+        <v>-0.3010588235294118</v>
+      </c>
+      <c r="J7" s="12" t="n">
+        <v>-0.234971264367816</v>
+      </c>
+      <c r="K7" s="12" t="n">
+        <v>-0.2409634551495017</v>
+      </c>
+      <c r="L7" s="12" t="n">
+        <v>-0.4715524193548387</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>-0.07771717171717177</v>
+      </c>
+      <c r="N7" s="12" t="n">
+        <v>-0.1990816326530613</v>
+      </c>
+      <c r="O7" s="5" t="n">
+        <v>0.01470588235294117</v>
+      </c>
+      <c r="P7" s="5" t="n">
+        <v>0.1155678670360112</v>
+      </c>
+      <c r="Q7" s="5" t="n">
+        <v>0.14295</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>BRINK Labor Hrs</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="G9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="K9" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="L9" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="M9" t="n">
+        <v>5.72</v>
+      </c>
+      <c r="N9" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="O9" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="P9" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>6</v>
+      </c>
+      <c r="R9" t="n">
+        <v>5.07</v>
+      </c>
+      <c r="S9" t="n">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>BRINK Labor $</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>12.53</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>39.75</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>39.75</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>18.45</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>51.25</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>51.25</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>51.25</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>52.48</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>64.38</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>49.73</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>68.34999999999999</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>73.84999999999999</v>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>78.25</v>
+      </c>
+      <c r="Q10" s="3" t="n">
+        <v>78.25</v>
+      </c>
+      <c r="R10" s="3" t="n">
+        <v>67.98</v>
+      </c>
+      <c r="S10" s="3" t="n">
+        <v>17.65</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>BRINK Labor %</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>100</v>
+      </c>
+      <c r="D11" t="n">
+        <v>100</v>
+      </c>
+      <c r="E11" t="n">
+        <v>100</v>
+      </c>
+      <c r="F11" t="n">
+        <v>100</v>
+      </c>
+      <c r="G11" t="n">
+        <v>24.13</v>
+      </c>
+      <c r="H11" t="n">
+        <v>18.35</v>
+      </c>
+      <c r="I11" t="n">
+        <v>21.57</v>
+      </c>
+      <c r="J11" t="n">
+        <v>19.71</v>
+      </c>
+      <c r="K11" t="n">
+        <v>28.18</v>
+      </c>
+      <c r="L11" t="n">
+        <v>18.97</v>
+      </c>
+      <c r="M11" t="n">
+        <v>14.61</v>
+      </c>
+      <c r="N11" t="n">
+        <v>17.42</v>
+      </c>
+      <c r="O11" t="n">
+        <v>12.97</v>
+      </c>
+      <c r="P11" t="n">
+        <v>19.43</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>34.23</v>
+      </c>
+      <c r="R11" t="n">
+        <v>100</v>
+      </c>
+      <c r="S11" t="n">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:S1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KY-2065 — 2026-04-20 — Teamworx Forecast vs Brink Actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>6AM</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>7AM</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>8AM</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>9AM</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>10AM</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>11AM</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>12PM</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>1PM</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>2PM</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>3PM</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>4PM</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>5PM</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>6PM</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>7PM</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>8PM</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>9PM</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>10PM</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>11PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>TWX FORECAST $</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>296</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>437</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>303</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>231</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>286</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>276</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>391</v>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>481</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>466</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>344</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>243</v>
+      </c>
+      <c r="R4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>BRINK ACTUAL $</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>153.18</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>434.29</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>170.54</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>239.76</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>307.56</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>289.3</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>447.8</v>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>602.65</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>411.72</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>308.26</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>71.3</v>
+      </c>
+      <c r="R5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>VARIANCE $ (Actual−Forecast)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>-142.82</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>-2.71</v>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>-132.46</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>8.76</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>21.56</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="M6" s="10" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="N6" s="10" t="n">
+        <v>121.65</v>
+      </c>
+      <c r="O6" s="11" t="n">
+        <v>-54.28</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>-35.74</v>
+      </c>
+      <c r="Q6" s="11" t="n">
+        <v>-171.7</v>
+      </c>
+      <c r="R6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>VARIANCE % (Δ/Forecast)</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="n">
+        <v>-0.4825</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>-0.006201372997711624</v>
+      </c>
+      <c r="I7" s="12" t="n">
+        <v>-0.4371617161716172</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>0.03792207792207788</v>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>0.0753846153846154</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>0.04818840579710149</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>0.1452685421994885</v>
+      </c>
+      <c r="N7" s="12" t="n">
+        <v>0.2529106029106029</v>
+      </c>
+      <c r="O7" s="5" t="n">
+        <v>-0.1164806866952789</v>
+      </c>
+      <c r="P7" s="5" t="n">
+        <v>-0.1038953488372093</v>
+      </c>
+      <c r="Q7" s="12" t="n">
+        <v>-0.7065843621399176</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>BRINK Labor Hrs</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" t="n">
+        <v>4</v>
+      </c>
+      <c r="I9" t="n">
+        <v>4</v>
+      </c>
+      <c r="J9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" t="n">
+        <v>4</v>
+      </c>
+      <c r="L9" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="M9" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="N9" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="O9" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="P9" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>7</v>
+      </c>
+      <c r="R9" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="S9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>BRINK Labor $</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>4.93</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>24.95</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>35.75</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>19.67</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>35.75</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>35.75</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>35.75</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>35.75</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>35.75</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>42.17</v>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>66.84999999999999</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>64.45</v>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>73.25</v>
+      </c>
+      <c r="Q10" s="3" t="n">
+        <v>73.25</v>
+      </c>
+      <c r="R10" s="3" t="n">
+        <v>63.94</v>
+      </c>
+      <c r="S10" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>BRINK Labor %</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>100</v>
+      </c>
+      <c r="D11" t="n">
+        <v>100</v>
+      </c>
+      <c r="E11" t="n">
+        <v>100</v>
+      </c>
+      <c r="F11" t="n">
+        <v>100</v>
+      </c>
+      <c r="G11" t="n">
+        <v>23.34</v>
+      </c>
+      <c r="H11" t="n">
+        <v>8.23</v>
+      </c>
+      <c r="I11" t="n">
+        <v>20.96</v>
+      </c>
+      <c r="J11" t="n">
+        <v>14.91</v>
+      </c>
+      <c r="K11" t="n">
+        <v>11.62</v>
+      </c>
+      <c r="L11" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="M11" t="n">
+        <v>9.42</v>
+      </c>
+      <c r="N11" t="n">
+        <v>11.09</v>
+      </c>
+      <c r="O11" t="n">
+        <v>15.65</v>
+      </c>
+      <c r="P11" t="n">
+        <v>23.76</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>102.73</v>
+      </c>
+      <c r="R11" t="n">
+        <v>100</v>
+      </c>
+      <c r="S11" t="n">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:S1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
           <t>KY-2065 — 2026-04-27 — Teamworx Forecast vs Brink Actual</t>
         </is>
       </c>

</xml_diff>